<commit_message>
2-2 Handout update in blue
</commit_message>
<xml_diff>
--- a/handouts/chapter_2_2_handout.xlsx
+++ b/handouts/chapter_2_2_handout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\craigaj\Documents\GitHub\timeseries\handouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{503E0F48-A0A6-4B33-9609-9D326196E843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A94151F9-1C8C-41BB-942B-57399B9900FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{CB73943A-C465-40BE-817C-B9991112161C}"/>
   </bookViews>
@@ -364,6 +364,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -372,15 +381,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6655,15 +6655,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="22" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="28"/>
     </row>
     <row r="2" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -6936,15 +6936,15 @@
       <c r="I13" s="7"/>
     </row>
     <row r="16" spans="1:9" s="22" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="23" t="s">
+      <c r="A16" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="25"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="28"/>
     </row>
     <row r="17" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
@@ -7035,15 +7035,15 @@
       <c r="B21" s="9">
         <v>4</v>
       </c>
-      <c r="C21" s="26"/>
+      <c r="C21" s="23"/>
       <c r="D21" s="4">
         <v>-0.7</v>
       </c>
       <c r="E21" s="4">
         <v>0.49</v>
       </c>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
@@ -7052,15 +7052,15 @@
       <c r="B22" s="10">
         <v>4.4000000000000004</v>
       </c>
-      <c r="C22" s="26"/>
+      <c r="C22" s="23"/>
       <c r="D22" s="4">
         <v>-0.3</v>
       </c>
       <c r="E22" s="4">
         <v>0.09</v>
       </c>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
@@ -7069,15 +7069,15 @@
       <c r="B23" s="11">
         <v>4.7</v>
       </c>
-      <c r="C23" s="26"/>
+      <c r="C23" s="23"/>
       <c r="D23" s="4">
         <v>0</v>
       </c>
       <c r="E23" s="4">
         <v>0</v>
       </c>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
@@ -7179,27 +7179,27 @@
       <c r="B28" s="19">
         <v>47</v>
       </c>
-      <c r="C28" s="27"/>
+      <c r="C28" s="24"/>
       <c r="D28" s="19">
         <v>0</v>
       </c>
       <c r="E28" s="19">
         <v>2.7</v>
       </c>
-      <c r="F28" s="27"/>
-      <c r="G28" s="28"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="25"/>
       <c r="I28" s="7"/>
     </row>
     <row r="31" spans="1:9" s="22" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="23" t="s">
+      <c r="A31" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B31" s="24"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="24"/>
-      <c r="G31" s="25"/>
+      <c r="B31" s="27"/>
+      <c r="C31" s="27"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="28"/>
     </row>
     <row r="32" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
@@ -7382,15 +7382,15 @@
       <c r="B40" s="13">
         <v>5.3</v>
       </c>
-      <c r="C40" s="26"/>
+      <c r="C40" s="23"/>
       <c r="D40" s="4">
         <v>0.6</v>
       </c>
       <c r="E40" s="4">
         <v>0.36</v>
       </c>
-      <c r="F40" s="26"/>
-      <c r="G40" s="26"/>
+      <c r="F40" s="23"/>
+      <c r="G40" s="23"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" s="4">
@@ -7399,15 +7399,15 @@
       <c r="B41" s="14">
         <v>5.4</v>
       </c>
-      <c r="C41" s="26"/>
+      <c r="C41" s="23"/>
       <c r="D41" s="4">
         <v>0.7</v>
       </c>
       <c r="E41" s="4">
         <v>0.49</v>
       </c>
-      <c r="F41" s="26"/>
-      <c r="G41" s="26"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="23"/>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" s="4">
@@ -7416,15 +7416,15 @@
       <c r="B42" s="5">
         <v>5.5</v>
       </c>
-      <c r="C42" s="26"/>
+      <c r="C42" s="23"/>
       <c r="D42" s="4">
         <v>0.8</v>
       </c>
       <c r="E42" s="4">
         <v>0.64</v>
       </c>
-      <c r="F42" s="26"/>
-      <c r="G42" s="26"/>
+      <c r="F42" s="23"/>
+      <c r="G42" s="23"/>
       <c r="I42" s="7"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
@@ -7452,15 +7452,15 @@
       <c r="I43" s="7"/>
     </row>
     <row r="46" spans="1:9" s="22" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A46" s="23" t="s">
+      <c r="A46" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B46" s="24"/>
-      <c r="C46" s="24"/>
-      <c r="D46" s="24"/>
-      <c r="E46" s="24"/>
-      <c r="F46" s="24"/>
-      <c r="G46" s="25"/>
+      <c r="B46" s="27"/>
+      <c r="C46" s="27"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="27"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="28"/>
     </row>
     <row r="47" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
@@ -7482,11 +7482,11 @@
       <c r="B48" s="5">
         <v>4.4000000000000004</v>
       </c>
-      <c r="C48" s="26"/>
-      <c r="D48" s="26"/>
-      <c r="E48" s="26"/>
-      <c r="F48" s="26"/>
-      <c r="G48" s="26"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="23"/>
+      <c r="E48" s="23"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="23"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" s="4">
@@ -7495,11 +7495,11 @@
       <c r="B49" s="6">
         <v>4.2</v>
       </c>
-      <c r="C49" s="26"/>
-      <c r="D49" s="26"/>
-      <c r="E49" s="26"/>
-      <c r="F49" s="26"/>
-      <c r="G49" s="26"/>
+      <c r="C49" s="23"/>
+      <c r="D49" s="23"/>
+      <c r="E49" s="23"/>
+      <c r="F49" s="23"/>
+      <c r="G49" s="23"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" s="4">
@@ -7508,11 +7508,11 @@
       <c r="B50" s="8">
         <v>4.2</v>
       </c>
-      <c r="C50" s="26"/>
-      <c r="D50" s="26"/>
-      <c r="E50" s="26"/>
-      <c r="F50" s="26"/>
-      <c r="G50" s="26"/>
+      <c r="C50" s="23"/>
+      <c r="D50" s="23"/>
+      <c r="E50" s="23"/>
+      <c r="F50" s="23"/>
+      <c r="G50" s="23"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" s="4">
@@ -7521,11 +7521,11 @@
       <c r="B51" s="9">
         <v>4</v>
       </c>
-      <c r="C51" s="26"/>
-      <c r="D51" s="26"/>
-      <c r="E51" s="26"/>
-      <c r="F51" s="26"/>
-      <c r="G51" s="26"/>
+      <c r="C51" s="23"/>
+      <c r="D51" s="23"/>
+      <c r="E51" s="23"/>
+      <c r="F51" s="23"/>
+      <c r="G51" s="23"/>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" s="4">
@@ -7534,11 +7534,11 @@
       <c r="B52" s="10">
         <v>4.4000000000000004</v>
       </c>
-      <c r="C52" s="26"/>
-      <c r="D52" s="26"/>
-      <c r="E52" s="26"/>
-      <c r="F52" s="26"/>
-      <c r="G52" s="26"/>
+      <c r="C52" s="23"/>
+      <c r="D52" s="23"/>
+      <c r="E52" s="23"/>
+      <c r="F52" s="23"/>
+      <c r="G52" s="23"/>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" s="4">
@@ -7547,11 +7547,11 @@
       <c r="B53" s="11">
         <v>4.7</v>
       </c>
-      <c r="C53" s="26"/>
-      <c r="D53" s="26"/>
-      <c r="E53" s="26"/>
-      <c r="F53" s="26"/>
-      <c r="G53" s="26"/>
+      <c r="C53" s="23"/>
+      <c r="D53" s="23"/>
+      <c r="E53" s="23"/>
+      <c r="F53" s="23"/>
+      <c r="G53" s="23"/>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" s="4">
@@ -7560,11 +7560,11 @@
       <c r="B54" s="12">
         <v>4.9000000000000004</v>
       </c>
-      <c r="C54" s="26"/>
-      <c r="D54" s="26"/>
-      <c r="E54" s="26"/>
-      <c r="F54" s="26"/>
-      <c r="G54" s="26"/>
+      <c r="C54" s="23"/>
+      <c r="D54" s="23"/>
+      <c r="E54" s="23"/>
+      <c r="F54" s="23"/>
+      <c r="G54" s="23"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" s="4">
@@ -7573,11 +7573,11 @@
       <c r="B55" s="13">
         <v>5.3</v>
       </c>
-      <c r="C55" s="26"/>
-      <c r="D55" s="26"/>
-      <c r="E55" s="26"/>
-      <c r="F55" s="26"/>
-      <c r="G55" s="26"/>
+      <c r="C55" s="23"/>
+      <c r="D55" s="23"/>
+      <c r="E55" s="23"/>
+      <c r="F55" s="23"/>
+      <c r="G55" s="23"/>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" s="4">
@@ -7586,11 +7586,11 @@
       <c r="B56" s="14">
         <v>5.4</v>
       </c>
-      <c r="C56" s="26"/>
-      <c r="D56" s="26"/>
-      <c r="E56" s="26"/>
-      <c r="F56" s="26"/>
-      <c r="G56" s="26"/>
+      <c r="C56" s="23"/>
+      <c r="D56" s="23"/>
+      <c r="E56" s="23"/>
+      <c r="F56" s="23"/>
+      <c r="G56" s="23"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" s="4">
@@ -7599,11 +7599,11 @@
       <c r="B57" s="5">
         <v>5.5</v>
       </c>
-      <c r="C57" s="26"/>
-      <c r="D57" s="26"/>
-      <c r="E57" s="26"/>
-      <c r="F57" s="26"/>
-      <c r="G57" s="26"/>
+      <c r="C57" s="23"/>
+      <c r="D57" s="23"/>
+      <c r="E57" s="23"/>
+      <c r="F57" s="23"/>
+      <c r="G57" s="23"/>
       <c r="I57" s="7"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.35">
@@ -7642,6 +7642,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010070F75838E79B0E48B83E8E3F5479A3A2" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2b0c304636f8f537543cd13f583db9d4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="ca1cba85-b018-40b2-9d9a-243cd5b6fae5" xmlns:ns4="f1fb8133-dfcb-4ab3-83e1-bcafde3f766a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f089f22c5ce4e61126931f7622145b2" ns3:_="" ns4:_="">
     <xsd:import namespace="ca1cba85-b018-40b2-9d9a-243cd5b6fae5"/>
@@ -7836,15 +7845,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5E1B631-90B0-4D19-A35E-F8DC8BE167A4}">
   <ds:schemaRefs>
@@ -7863,6 +7863,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDDC771-C014-4A48-9FCA-802C556EA1D0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7879,12 +7887,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C96E0334-A0AA-41B5-AE21-CAD1C9D10746}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>